<commit_message>
DoeRunner Excel Pfad angepasst suiii
</commit_message>
<xml_diff>
--- a/GA_Gruppierung_Test04.03.2026/layouts_with_machines.xlsx
+++ b/GA_Gruppierung_Test04.03.2026/layouts_with_machines.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carey\OneDrive\Bachelorarbeit\BA-Code\GA_Gruppierung_Test04.03.2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6908A1B4-506B-4559-BC06-B1B2FCBCCB73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1299B01B-770B-47E8-B0D5-24DD3F84D490}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="9" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Vorlage" sheetId="10" r:id="rId1"/>
@@ -3746,7 +3746,7 @@
         <v>0</v>
       </c>
       <c r="E2" s="4">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="F2" s="4">
         <v>0</v>
@@ -3771,16 +3771,16 @@
         <v>17</v>
       </c>
       <c r="C3" s="4">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="D3" s="4">
         <v>0</v>
       </c>
       <c r="E3" s="4">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="F3" s="4">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>
@@ -3802,16 +3802,16 @@
         <v>17</v>
       </c>
       <c r="C4" s="4">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="D4" s="4">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="E4" s="4">
         <v>0</v>
       </c>
       <c r="F4" s="4">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -3836,7 +3836,7 @@
         <v>0</v>
       </c>
       <c r="D5" s="4">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="E5" s="4">
         <v>0</v>

</xml_diff>

<commit_message>
Inkonisstente Material und Worker Punkte
</commit_message>
<xml_diff>
--- a/GA_Gruppierung_Test04.03.2026/layouts_with_machines.xlsx
+++ b/GA_Gruppierung_Test04.03.2026/layouts_with_machines.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carey\OneDrive\Bachelorarbeit\BA-Code\GA_Gruppierung_Test04.03.2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1299B01B-770B-47E8-B0D5-24DD3F84D490}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40CB1676-C31B-4B83-8A8D-1B8D4E86E711}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="9" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2724" yWindow="2724" windowWidth="17280" windowHeight="8340" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Vorlage" sheetId="10" r:id="rId1"/>
@@ -3913,13 +3913,13 @@
         <v>25</v>
       </c>
       <c r="O7" s="8">
-        <v>1</v>
+        <v>1.9</v>
       </c>
       <c r="P7" s="12" t="s">
         <v>26</v>
       </c>
       <c r="Q7" s="8">
-        <v>1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="R7" s="8">
         <v>1</v>
@@ -3928,7 +3928,7 @@
         <v>28</v>
       </c>
       <c r="T7" s="8">
-        <v>2</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="8" spans="1:26" x14ac:dyDescent="0.3">
@@ -3961,13 +3961,13 @@
         <v>25</v>
       </c>
       <c r="O8" s="8">
-        <v>1</v>
+        <v>1.05</v>
       </c>
       <c r="P8" s="12" t="s">
         <v>26</v>
       </c>
       <c r="Q8" s="8">
-        <v>1</v>
+        <v>1.95</v>
       </c>
       <c r="R8" s="8">
         <v>2</v>
@@ -3976,7 +3976,7 @@
         <v>25</v>
       </c>
       <c r="T8" s="8">
-        <v>2</v>
+        <v>2.0499999999999998</v>
       </c>
     </row>
     <row r="9" spans="1:26" x14ac:dyDescent="0.3">
@@ -4009,13 +4009,13 @@
         <v>26</v>
       </c>
       <c r="O9" s="8">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="P9" s="12" t="s">
         <v>28</v>
       </c>
       <c r="Q9" s="8">
-        <v>1</v>
+        <v>1.8</v>
       </c>
       <c r="R9" s="8">
         <v>1</v>
@@ -4024,7 +4024,7 @@
         <v>27</v>
       </c>
       <c r="T9" s="8">
-        <v>2</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="10" spans="1:26" x14ac:dyDescent="0.3">
@@ -4057,13 +4057,13 @@
         <v>27</v>
       </c>
       <c r="O10" s="8">
-        <v>1</v>
+        <v>1.05</v>
       </c>
       <c r="P10" s="12" t="s">
         <v>26</v>
       </c>
       <c r="Q10" s="8">
-        <v>1</v>
+        <v>2.95</v>
       </c>
       <c r="R10" s="8">
         <v>2</v>
@@ -4072,7 +4072,7 @@
         <v>26</v>
       </c>
       <c r="T10" s="8">
-        <v>2</v>
+        <v>2.95</v>
       </c>
     </row>
     <row r="11" spans="1:26" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Tauschen veralgemeinert, teleport hinzugefügt, corssover abhängig von Wahrscheinlichkeit, abbruch abhängig von Kriterien
</commit_message>
<xml_diff>
--- a/GA_Gruppierung_Test04.03.2026/layouts_with_machines.xlsx
+++ b/GA_Gruppierung_Test04.03.2026/layouts_with_machines.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carey\OneDrive\Bachelorarbeit\BA-Code\GA_Gruppierung_Test04.03.2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40CB1676-C31B-4B83-8A8D-1B8D4E86E711}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{907BE74F-2BEB-4646-B85E-B546D49DB80C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2724" yWindow="2724" windowWidth="17280" windowHeight="8340" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Vorlage" sheetId="10" r:id="rId1"/>
@@ -3746,7 +3746,7 @@
         <v>0</v>
       </c>
       <c r="E2" s="4">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F2" s="4">
         <v>0</v>
@@ -3771,16 +3771,16 @@
         <v>17</v>
       </c>
       <c r="C3" s="4">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="D3" s="4">
         <v>0</v>
       </c>
       <c r="E3" s="4">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F3" s="4">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>
@@ -3802,16 +3802,16 @@
         <v>17</v>
       </c>
       <c r="C4" s="4">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D4" s="4">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="E4" s="4">
         <v>0</v>
       </c>
       <c r="F4" s="4">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -3836,7 +3836,7 @@
         <v>0</v>
       </c>
       <c r="D5" s="4">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="E5" s="4">
         <v>0</v>

</xml_diff>